<commit_message>
Rectified the pregnancy form calculation
</commit_message>
<xml_diff>
--- a/forms/app/pregnancy_counselling.xlsx
+++ b/forms/app/pregnancy_counselling.xlsx
@@ -1000,12 +1000,6 @@
     <t>${high_risk_manual}  = "false"  and ${is_high_risk_pregnancy_ML} = "true"</t>
   </si>
   <si>
-    <t>${high_risk_manual}  = "true"  and ${is_high_risk_pregnancy_ML} = "true"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">begin repeat </t>
-  </si>
-  <si>
     <t xml:space="preserve">questions_to_client </t>
   </si>
   <si>
@@ -1021,9 +1015,6 @@
     <t>current_name</t>
   </si>
   <si>
-    <t xml:space="preserve">end repeat </t>
-  </si>
-  <si>
     <t>imran</t>
   </si>
   <si>
@@ -1034,6 +1025,15 @@
   </si>
   <si>
     <t>indexed-repeat(${esmail}, ${imran}, position(..))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">begin_repeat </t>
+  </si>
+  <si>
+    <t xml:space="preserve">end_repeat </t>
+  </si>
+  <si>
+    <t>${high_risk_manual}  = "true"  or  ${is_high_risk_pregnancy_ML} = "true"</t>
   </si>
 </sst>
 </file>
@@ -1465,7 +1465,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>4</v>
@@ -5025,7 +5025,7 @@
         <v>202</v>
       </c>
       <c r="G122" s="26" t="s">
-        <v>315</v>
+        <v>326</v>
       </c>
       <c r="H122" t="s">
         <v>125</v>
@@ -5044,10 +5044,10 @@
     </row>
     <row r="124" spans="1:14" s="37" customFormat="1">
       <c r="A124" s="16" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="B124" s="16" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="E124" s="37">
         <v>1</v>
@@ -5058,55 +5058,54 @@
         <v>41</v>
       </c>
       <c r="B125" s="16" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="M125" s="37" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
     </row>
     <row r="126" spans="1:14" s="37" customFormat="1">
       <c r="A126" s="16" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B126" s="16" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="127" spans="1:14" s="29" customFormat="1">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="127" spans="1:14" s="37" customFormat="1">
       <c r="A127" s="16" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="B127" s="16" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="E127" s="26" t="s">
-        <v>320</v>
-      </c>
-      <c r="H127" s="29" t="s">
+        <v>318</v>
+      </c>
+      <c r="H127" s="37" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="128" spans="1:14" s="29" customFormat="1">
+    <row r="128" spans="1:14" s="37" customFormat="1">
       <c r="A128" s="27" t="s">
         <v>41</v>
       </c>
       <c r="B128" s="27" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="M128" s="26" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="129" spans="1:8" s="25" customFormat="1">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" s="37" customFormat="1">
       <c r="A129" s="16" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B129" s="16" t="s">
-        <v>318</v>
-      </c>
-      <c r="E129" s="29"/>
-    </row>
-    <row r="130" spans="1:8">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8" s="37" customFormat="1">
       <c r="A130" s="16" t="s">
         <v>99</v>
       </c>

</xml_diff>

<commit_message>
Added qn mark to mitigation questions
</commit_message>
<xml_diff>
--- a/forms/app/pregnancy_counselling.xlsx
+++ b/forms/app/pregnancy_counselling.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="498">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1482" uniqueCount="499">
   <si>
     <t>type</t>
   </si>
@@ -1149,82 +1149,40 @@
     <t>mitigation_note_1</t>
   </si>
   <si>
-    <t xml:space="preserve">Do you understand the importance of Facility Delivery </t>
-  </si>
-  <si>
-    <t>Je unaelewa umuhimu wa Kujifungulia kituo cha afya</t>
-  </si>
-  <si>
     <t>contains(${mitigation_list},”facility_delivery“)</t>
   </si>
   <si>
     <t>mitigation_note_2</t>
   </si>
   <si>
-    <t xml:space="preserve">Do you understand the importance of ANC Visits </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Je unaelewa umuhimu wa Kuhudhuria kliniki wakati wa ujauzito </t>
-  </si>
-  <si>
     <t>contains(${mitigation_list},”anc_visits“)</t>
   </si>
   <si>
     <t>mitigation_note_3</t>
   </si>
   <si>
-    <t>Do you understand the importance of Rest</t>
-  </si>
-  <si>
-    <t>Je unaelewa umuhimu wa Kupumzika</t>
-  </si>
-  <si>
     <t>contains(${mitigation_list},”rest“)</t>
   </si>
   <si>
     <t>mitigation_note_4</t>
   </si>
   <si>
-    <t xml:space="preserve">Do you understand the importance of Balanced Diet/Good Nutrition Practices </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Je unaelewa umuhimu wa Kula vyakula vyenye virutubisho </t>
-  </si>
-  <si>
     <t>contains(${mitigation_list},”balanced_diet“)</t>
   </si>
   <si>
     <t>mitigation_note_5</t>
   </si>
   <si>
-    <t xml:space="preserve">Do you understand the importance of No heavy work </t>
-  </si>
-  <si>
-    <t>Je unaelewa umuhimu wa Kutokufanya kazi ngumu</t>
-  </si>
-  <si>
     <t>contains(${mitigation_list},”no_heavy_work “)</t>
   </si>
   <si>
     <t>mitigation_note_6</t>
   </si>
   <si>
-    <t xml:space="preserve">Do you understand the importance of Family Planning </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Je unaelewa umuhimu wa Kutumia uzazi wa mpango </t>
-  </si>
-  <si>
     <t>contains(${mitigation_list},”family_planning“)</t>
   </si>
   <si>
     <t>mitigation_note_7</t>
-  </si>
-  <si>
-    <t>Do you understand the importance of Risks of using herbs</t>
-  </si>
-  <si>
-    <t>Je unaelewa umuhimu wa Hatari za kutumia dawa za mitishamba</t>
   </si>
   <si>
     <t>contains(${mitigation_list},”local_herbs_risks“)</t>
@@ -1574,13 +1532,58 @@
   </si>
   <si>
     <t>Milalo mibaya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you understand the importance of Facility Delivery ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you understand the importance of ANC Visits ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you understand the importance of Rest ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you understand the importance of Balanced Diet/Good Nutrition Practices  ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you understand the importance of No heavy work  ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you understand the importance of Family Planning  ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you understand the importance of Risks of using herbs ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mkakati wa kuepuka sababu za hatari za ujauzito ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je unaelewa umuhimu wa Kujifungulia kituo cha afya ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je unaelewa umuhimu wa Kuhudhuria kliniki wakati wa ujauzito  ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je unaelewa umuhimu wa Kupumzika ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je unaelewa umuhimu wa Kula vyakula vyenye virutubisho  ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je unaelewa umuhimu wa Kutokufanya kazi ngumu ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je unaelewa umuhimu wa Kutumia uzazi wa mpango ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je unaelewa umuhimu wa Hatari za kutumia dawa za mitishamba ? </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1649,6 +1652,12 @@
       <name val="Cambria"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1697,7 +1706,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -1753,6 +1762,7 @@
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5921,7 +5931,7 @@
         <v>290</v>
       </c>
       <c r="D120" t="s">
-        <v>497</v>
+        <v>483</v>
       </c>
       <c r="G120" s="21" t="s">
         <v>291</v>
@@ -6272,7 +6282,7 @@
         <v>337</v>
       </c>
       <c r="D142" s="5" t="s">
-        <v>338</v>
+        <v>491</v>
       </c>
       <c r="G142" s="5" t="s">
         <v>355</v>
@@ -6285,15 +6295,15 @@
       <c r="B143" t="s">
         <v>356</v>
       </c>
-      <c r="C143" t="s">
-        <v>357</v>
-      </c>
-      <c r="D143" t="s">
-        <v>358</v>
+      <c r="C143" s="29" t="s">
+        <v>484</v>
+      </c>
+      <c r="D143" s="29" t="s">
+        <v>492</v>
       </c>
       <c r="E143"/>
       <c r="G143" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="144" spans="1:14">
@@ -6301,17 +6311,17 @@
         <v>116</v>
       </c>
       <c r="B144" t="s">
-        <v>360</v>
-      </c>
-      <c r="C144" t="s">
-        <v>361</v>
-      </c>
-      <c r="D144" t="s">
-        <v>362</v>
+        <v>358</v>
+      </c>
+      <c r="C144" s="29" t="s">
+        <v>485</v>
+      </c>
+      <c r="D144" s="29" t="s">
+        <v>493</v>
       </c>
       <c r="E144"/>
       <c r="G144" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
     </row>
     <row r="145" spans="1:27">
@@ -6319,17 +6329,17 @@
         <v>116</v>
       </c>
       <c r="B145" t="s">
-        <v>364</v>
-      </c>
-      <c r="C145" t="s">
-        <v>365</v>
-      </c>
-      <c r="D145" t="s">
-        <v>366</v>
+        <v>360</v>
+      </c>
+      <c r="C145" s="29" t="s">
+        <v>486</v>
+      </c>
+      <c r="D145" s="29" t="s">
+        <v>494</v>
       </c>
       <c r="E145"/>
       <c r="G145" t="s">
-        <v>367</v>
+        <v>361</v>
       </c>
     </row>
     <row r="146" spans="1:27">
@@ -6337,17 +6347,17 @@
         <v>116</v>
       </c>
       <c r="B146" t="s">
-        <v>368</v>
-      </c>
-      <c r="C146" t="s">
-        <v>369</v>
-      </c>
-      <c r="D146" t="s">
-        <v>370</v>
+        <v>362</v>
+      </c>
+      <c r="C146" s="29" t="s">
+        <v>487</v>
+      </c>
+      <c r="D146" s="29" t="s">
+        <v>495</v>
       </c>
       <c r="E146"/>
       <c r="G146" t="s">
-        <v>371</v>
+        <v>363</v>
       </c>
     </row>
     <row r="147" spans="1:27">
@@ -6355,17 +6365,17 @@
         <v>116</v>
       </c>
       <c r="B147" t="s">
-        <v>372</v>
-      </c>
-      <c r="C147" t="s">
-        <v>373</v>
-      </c>
-      <c r="D147" t="s">
-        <v>374</v>
+        <v>364</v>
+      </c>
+      <c r="C147" s="29" t="s">
+        <v>488</v>
+      </c>
+      <c r="D147" s="29" t="s">
+        <v>496</v>
       </c>
       <c r="E147"/>
       <c r="G147" t="s">
-        <v>375</v>
+        <v>365</v>
       </c>
     </row>
     <row r="148" spans="1:27">
@@ -6373,17 +6383,17 @@
         <v>116</v>
       </c>
       <c r="B148" t="s">
-        <v>376</v>
-      </c>
-      <c r="C148" t="s">
-        <v>377</v>
-      </c>
-      <c r="D148" t="s">
-        <v>378</v>
+        <v>366</v>
+      </c>
+      <c r="C148" s="29" t="s">
+        <v>489</v>
+      </c>
+      <c r="D148" s="29" t="s">
+        <v>497</v>
       </c>
       <c r="E148"/>
       <c r="G148" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
     </row>
     <row r="149" spans="1:27">
@@ -6391,17 +6401,17 @@
         <v>116</v>
       </c>
       <c r="B149" t="s">
-        <v>380</v>
-      </c>
-      <c r="C149" t="s">
-        <v>381</v>
-      </c>
-      <c r="D149" t="s">
-        <v>382</v>
+        <v>368</v>
+      </c>
+      <c r="C149" s="29" t="s">
+        <v>490</v>
+      </c>
+      <c r="D149" s="29" t="s">
+        <v>498</v>
       </c>
       <c r="E149"/>
       <c r="G149" t="s">
-        <v>383</v>
+        <v>369</v>
       </c>
     </row>
     <row r="150" spans="1:27" s="2" customFormat="1">
@@ -6418,13 +6428,13 @@
         <v>112</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>384</v>
+        <v>370</v>
       </c>
       <c r="C151" t="s">
-        <v>385</v>
+        <v>371</v>
       </c>
       <c r="D151" t="s">
-        <v>386</v>
+        <v>372</v>
       </c>
       <c r="H151" t="s">
         <v>237</v>
@@ -6436,17 +6446,17 @@
         <v>116</v>
       </c>
       <c r="B152" s="13" t="s">
-        <v>387</v>
+        <v>373</v>
       </c>
       <c r="C152" s="13" t="s">
-        <v>388</v>
+        <v>374</v>
       </c>
       <c r="D152" s="15" t="s">
-        <v>389</v>
+        <v>375</v>
       </c>
       <c r="E152" s="13"/>
       <c r="G152" s="13" t="s">
-        <v>390</v>
+        <v>376</v>
       </c>
       <c r="H152" s="13"/>
       <c r="I152" s="13"/>
@@ -6473,20 +6483,20 @@
         <v>116</v>
       </c>
       <c r="B153" s="13" t="s">
-        <v>391</v>
+        <v>377</v>
       </c>
       <c r="C153" s="13" t="s">
-        <v>392</v>
+        <v>378</v>
       </c>
       <c r="D153" s="23" t="s">
-        <v>393</v>
+        <v>379</v>
       </c>
       <c r="E153" s="13"/>
       <c r="G153" s="14" t="s">
-        <v>394</v>
+        <v>380</v>
       </c>
       <c r="H153" s="13" t="s">
-        <v>395</v>
+        <v>381</v>
       </c>
       <c r="I153" s="13"/>
       <c r="J153" s="13"/>
@@ -6512,20 +6522,20 @@
         <v>116</v>
       </c>
       <c r="B154" s="13" t="s">
-        <v>396</v>
+        <v>382</v>
       </c>
       <c r="C154" s="13" t="s">
-        <v>397</v>
+        <v>383</v>
       </c>
       <c r="D154" s="13" t="s">
-        <v>398</v>
+        <v>384</v>
       </c>
       <c r="E154" s="13"/>
       <c r="G154" s="24" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="H154" s="13" t="s">
-        <v>395</v>
+        <v>381</v>
       </c>
       <c r="I154" s="13"/>
       <c r="J154" s="13"/>
@@ -6551,13 +6561,13 @@
         <v>116</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>400</v>
+        <v>386</v>
       </c>
       <c r="C155" t="s">
-        <v>401</v>
+        <v>387</v>
       </c>
       <c r="D155" t="s">
-        <v>402</v>
+        <v>388</v>
       </c>
     </row>
     <row r="156" spans="1:27">
@@ -6565,7 +6575,7 @@
         <v>120</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>384</v>
+        <v>370</v>
       </c>
       <c r="K156" s="13"/>
     </row>
@@ -6574,7 +6584,7 @@
         <v>46</v>
       </c>
       <c r="B157" s="13" t="s">
-        <v>403</v>
+        <v>389</v>
       </c>
       <c r="C157" s="13"/>
       <c r="D157" s="13"/>
@@ -6585,7 +6595,7 @@
       <c r="I157" s="13"/>
       <c r="J157" s="13"/>
       <c r="M157" s="13" t="s">
-        <v>404</v>
+        <v>390</v>
       </c>
       <c r="N157" s="13"/>
       <c r="O157" s="13"/>
@@ -6607,10 +6617,10 @@
         <v>46</v>
       </c>
       <c r="B158" s="22" t="s">
-        <v>405</v>
+        <v>391</v>
       </c>
       <c r="M158" s="22" t="s">
-        <v>406</v>
+        <v>392</v>
       </c>
     </row>
     <row r="159" spans="1:27" s="2" customFormat="1">
@@ -6618,10 +6628,10 @@
         <v>46</v>
       </c>
       <c r="B159" s="22" t="s">
-        <v>407</v>
+        <v>393</v>
       </c>
       <c r="M159" s="22" t="s">
-        <v>408</v>
+        <v>394</v>
       </c>
     </row>
     <row r="160" spans="1:27" s="2" customFormat="1">
@@ -6629,11 +6639,11 @@
         <v>46</v>
       </c>
       <c r="B160" s="22" t="s">
-        <v>409</v>
+        <v>395</v>
       </c>
       <c r="K160"/>
       <c r="M160" s="22" t="s">
-        <v>410</v>
+        <v>396</v>
       </c>
     </row>
   </sheetData>
@@ -6659,7 +6669,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1">
       <c r="A1" s="25" t="s">
-        <v>411</v>
+        <v>397</v>
       </c>
       <c r="B1" s="25" t="s">
         <v>1</v>
@@ -6700,7 +6710,7 @@
         <v>230</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>412</v>
+        <v>398</v>
       </c>
       <c r="C2" s="26" t="s">
         <v>239</v>
@@ -6850,7 +6860,7 @@
         <v>255</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>413</v>
+        <v>399</v>
       </c>
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
@@ -7174,7 +7184,7 @@
         <v>290</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>497</v>
+        <v>483</v>
       </c>
       <c r="E15" s="13"/>
       <c r="F15" s="13"/>
@@ -7420,7 +7430,7 @@
         <v>230</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>414</v>
+        <v>400</v>
       </c>
       <c r="C22" s="15" t="s">
         <v>317</v>
@@ -7564,7 +7574,7 @@
         <v>230</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>415</v>
+        <v>401</v>
       </c>
       <c r="C26" s="15" t="s">
         <v>333</v>
@@ -7597,128 +7607,128 @@
     </row>
     <row r="27" spans="1:26" ht="15.75" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>416</v>
+        <v>402</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>417</v>
+        <v>403</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>418</v>
+        <v>404</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>419</v>
+        <v>405</v>
       </c>
     </row>
     <row r="28" spans="1:26" ht="15.75" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>416</v>
+        <v>402</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>420</v>
+        <v>406</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>421</v>
+        <v>407</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>422</v>
+        <v>408</v>
       </c>
     </row>
     <row r="29" spans="1:26" ht="15.75" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>416</v>
+        <v>402</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>423</v>
+        <v>409</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>424</v>
+        <v>410</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>425</v>
+        <v>411</v>
       </c>
     </row>
     <row r="30" spans="1:26" ht="15.75" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>416</v>
+        <v>402</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>426</v>
+        <v>412</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>427</v>
+        <v>413</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>428</v>
+        <v>414</v>
       </c>
     </row>
     <row r="31" spans="1:26" ht="15.75" customHeight="1">
       <c r="A31" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>416</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>430</v>
-      </c>
       <c r="D31" s="5" t="s">
-        <v>431</v>
+        <v>417</v>
       </c>
     </row>
     <row r="32" spans="1:26" ht="15.75" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>416</v>
+        <v>402</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>432</v>
+        <v>418</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>433</v>
+        <v>419</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>434</v>
+        <v>420</v>
       </c>
     </row>
     <row r="33" spans="1:26" ht="15.75" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>416</v>
+        <v>402</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>435</v>
+        <v>421</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>436</v>
+        <v>422</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>437</v>
+        <v>423</v>
       </c>
     </row>
     <row r="34" spans="1:26" ht="15.75" customHeight="1">
       <c r="A34" s="5" t="s">
-        <v>438</v>
+        <v>424</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>153</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>439</v>
+        <v>425</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>440</v>
+        <v>426</v>
       </c>
     </row>
     <row r="35" spans="1:26">
       <c r="A35" s="5" t="s">
-        <v>438</v>
+        <v>424</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>441</v>
+        <v>427</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>442</v>
+        <v>428</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>443</v>
+        <v>429</v>
       </c>
     </row>
     <row r="36" spans="1:26">
@@ -7726,13 +7736,13 @@
         <v>195</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>444</v>
+        <v>430</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>445</v>
+        <v>431</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>446</v>
+        <v>432</v>
       </c>
       <c r="E36" s="13"/>
       <c r="F36" s="13"/>
@@ -7762,13 +7772,13 @@
         <v>195</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>447</v>
+        <v>433</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>448</v>
+        <v>434</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>449</v>
+        <v>435</v>
       </c>
       <c r="E37" s="13"/>
       <c r="F37" s="13"/>
@@ -7798,13 +7808,13 @@
         <v>195</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>450</v>
+        <v>436</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>451</v>
+        <v>437</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>452</v>
+        <v>438</v>
       </c>
       <c r="E38" s="13"/>
       <c r="F38" s="13"/>
@@ -7834,13 +7844,13 @@
         <v>195</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>453</v>
+        <v>439</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>454</v>
+        <v>440</v>
       </c>
       <c r="D39" s="15" t="s">
-        <v>455</v>
+        <v>441</v>
       </c>
       <c r="E39" s="13"/>
       <c r="F39" s="13"/>
@@ -7870,13 +7880,13 @@
         <v>195</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>456</v>
+        <v>442</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>457</v>
+        <v>443</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>458</v>
+        <v>444</v>
       </c>
       <c r="E40" s="13"/>
       <c r="F40" s="13"/>
@@ -7906,13 +7916,13 @@
         <v>195</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>459</v>
+        <v>445</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>460</v>
+        <v>446</v>
       </c>
       <c r="D41" s="15" t="s">
-        <v>461</v>
+        <v>447</v>
       </c>
       <c r="E41" s="13"/>
       <c r="F41" s="13"/>
@@ -7942,13 +7952,13 @@
         <v>195</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>462</v>
+        <v>448</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>463</v>
+        <v>449</v>
       </c>
       <c r="D42" s="15" t="s">
-        <v>464</v>
+        <v>450</v>
       </c>
       <c r="E42" s="13"/>
       <c r="F42" s="13"/>
@@ -7978,13 +7988,13 @@
         <v>195</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>465</v>
+        <v>451</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>466</v>
+        <v>452</v>
       </c>
       <c r="D43" s="15" t="s">
-        <v>467</v>
+        <v>453</v>
       </c>
       <c r="E43" s="13"/>
       <c r="F43" s="13"/>
@@ -8014,13 +8024,13 @@
         <v>195</v>
       </c>
       <c r="B44" s="13" t="s">
-        <v>468</v>
+        <v>454</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>469</v>
+        <v>455</v>
       </c>
       <c r="D44" s="15" t="s">
-        <v>470</v>
+        <v>456</v>
       </c>
       <c r="E44" s="13"/>
       <c r="F44" s="13"/>
@@ -8050,13 +8060,13 @@
         <v>195</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>471</v>
+        <v>457</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>472</v>
+        <v>458</v>
       </c>
       <c r="D45" s="15" t="s">
-        <v>473</v>
+        <v>459</v>
       </c>
       <c r="E45" s="13"/>
       <c r="F45" s="13"/>
@@ -8086,13 +8096,13 @@
         <v>195</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>474</v>
+        <v>460</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>475</v>
+        <v>461</v>
       </c>
       <c r="D46" s="15" t="s">
-        <v>476</v>
+        <v>462</v>
       </c>
       <c r="E46" s="13"/>
       <c r="F46" s="13"/>
@@ -8122,13 +8132,13 @@
         <v>195</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>477</v>
+        <v>463</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>478</v>
+        <v>464</v>
       </c>
       <c r="D47" s="15" t="s">
-        <v>479</v>
+        <v>465</v>
       </c>
       <c r="E47" s="13"/>
       <c r="F47" s="13"/>
@@ -8158,13 +8168,13 @@
         <v>195</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>480</v>
+        <v>466</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>481</v>
+        <v>467</v>
       </c>
       <c r="D48" s="15" t="s">
-        <v>482</v>
+        <v>468</v>
       </c>
       <c r="E48" s="13"/>
       <c r="F48" s="13"/>
@@ -8194,13 +8204,13 @@
         <v>195</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>483</v>
+        <v>469</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>484</v>
+        <v>470</v>
       </c>
       <c r="D49" s="15" t="s">
-        <v>485</v>
+        <v>471</v>
       </c>
       <c r="E49" s="13"/>
       <c r="F49" s="13"/>
@@ -8243,22 +8253,22 @@
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1">
       <c r="A1" s="25" t="s">
-        <v>486</v>
+        <v>472</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>487</v>
+        <v>473</v>
       </c>
       <c r="C1" s="25" t="s">
-        <v>488</v>
+        <v>474</v>
       </c>
       <c r="D1" s="25" t="s">
-        <v>489</v>
+        <v>475</v>
       </c>
       <c r="E1" s="25" t="s">
-        <v>490</v>
+        <v>476</v>
       </c>
       <c r="F1" s="25" t="s">
-        <v>491</v>
+        <v>477</v>
       </c>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
@@ -8283,19 +8293,19 @@
     </row>
     <row r="2" spans="1:26" ht="15.75" customHeight="1">
       <c r="A2" s="20" t="s">
-        <v>492</v>
+        <v>478</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>493</v>
+        <v>479</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>494</v>
+        <v>480</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>495</v>
+        <v>481</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>496</v>
+        <v>482</v>
       </c>
       <c r="F2" s="20"/>
       <c r="G2" s="2"/>

</xml_diff>

<commit_message>
Rectified swahili translation for big baby
</commit_message>
<xml_diff>
--- a/forms/app/pregnancy_counselling.xlsx
+++ b/forms/app/pregnancy_counselling.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6620" tabRatio="500"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="5300" tabRatio="384"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="874" uniqueCount="511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="874" uniqueCount="516">
   <si>
     <t>type</t>
   </si>
@@ -1171,9 +1171,6 @@
     <t>mitigation_qn</t>
   </si>
   <si>
-    <t xml:space="preserve">Mkakati wa kuepuka sababu za hatari za ujauzito ? </t>
-  </si>
-  <si>
     <t>(${high_risk_manual}  = "true"  or  ${is_high_risk_pregnancy_ML} = "true") and ${emergency_danger_sign_referral} = 0</t>
   </si>
   <si>
@@ -1614,13 +1611,37 @@
   </si>
   <si>
     <t>../inputs/gestation_in_weeks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kifafa cha mimba
+Mama akipata tatizo hili hukutika mfano wa homa ya mdudu na kupoteza faham, kifafa cha mimba hutokea kabla au baada ya mama kujifungua. 
+</t>
+  </si>
+  <si>
+    <t>Milalo mibaya
+Kutokea akiwa na mlalo usio wa kawaida wakati wa mtoto kuzaliwa</t>
+  </si>
+  <si>
+    <t>Mtoto kutanguliza makalio 
+Mtoto kutokeza makalio wakati wa kuzaliwa kawaida atokee kichwa ili azae salama.</t>
+  </si>
+  <si>
+    <t>Seli mundu 
+Maradhi ya homa ya mifupa/seli nundu, mwenye maradhi haya chembe chembe nyekundu za damu huwa kidogo na hazikukamilika, hupekelea kuwa na ukosefu wa damu mara kwa mara</t>
+  </si>
+  <si>
+    <t>Maradhi ya moyo 
+Haya ni maradhi sugu ambapo moyo hushindwa kufanya kazi vizuri na tujuwe kwamba moyo ni kiungo kinacho sambaza damu safi kwenda sehemu zote za mwili</t>
+  </si>
+  <si>
+    <t>Mkakati wa kuepuka sababu za hatari za ujauzito</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1636,18 +1657,18 @@
     <font>
       <sz val="11"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1685,7 +1706,7 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1696,7 +1717,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1709,10 +1730,16 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -1749,7 +1776,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -1812,8 +1839,11 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2301,10 +2331,10 @@
         <v>25</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>507</v>
+      </c>
+      <c r="C4" s="34" t="s">
         <v>508</v>
-      </c>
-      <c r="C4" s="35" t="s">
-        <v>509</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -3271,14 +3301,14 @@
       <c r="I36" s="4"/>
       <c r="J36" s="4"/>
       <c r="K36" s="4"/>
-      <c r="L36" s="34" t="s">
+      <c r="L36" s="35" t="s">
         <v>75</v>
       </c>
-      <c r="M36" s="34"/>
-      <c r="N36" s="34"/>
-      <c r="O36" s="34"/>
-      <c r="P36" s="34"/>
-      <c r="Q36" s="34"/>
+      <c r="M36" s="35"/>
+      <c r="N36" s="35"/>
+      <c r="O36" s="35"/>
+      <c r="P36" s="35"/>
+      <c r="Q36" s="35"/>
       <c r="R36" s="5"/>
       <c r="S36" s="5"/>
       <c r="T36" s="5"/>
@@ -4009,7 +4039,7 @@
         <v>115</v>
       </c>
       <c r="L58" s="14" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="59" spans="1:26">
@@ -5033,7 +5063,7 @@
       <c r="Z92" s="18"/>
       <c r="AMJ92"/>
     </row>
-    <row r="93" spans="1:1024" s="15" customFormat="1" ht="65">
+    <row r="93" spans="1:1024" s="15" customFormat="1" ht="52">
       <c r="A93" s="18" t="s">
         <v>19</v>
       </c>
@@ -5490,7 +5520,7 @@
       <c r="Z104" s="18"/>
       <c r="AMJ104"/>
     </row>
-    <row r="105" spans="1:1024" s="15" customFormat="1" ht="117">
+    <row r="105" spans="1:1024" s="15" customFormat="1" ht="78">
       <c r="A105" s="18" t="s">
         <v>110</v>
       </c>
@@ -5941,7 +5971,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="121" spans="1:26">
+    <row r="121" spans="1:26" ht="65">
       <c r="A121" s="15" t="s">
         <v>110</v>
       </c>
@@ -5951,8 +5981,8 @@
       <c r="C121" s="15" t="s">
         <v>283</v>
       </c>
-      <c r="D121" s="14" t="s">
-        <v>185</v>
+      <c r="D121" s="18" t="s">
+        <v>510</v>
       </c>
       <c r="F121" s="27" t="s">
         <v>284</v>
@@ -6009,7 +6039,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="125" spans="1:26">
+    <row r="125" spans="1:26" ht="39">
       <c r="A125" s="15" t="s">
         <v>110</v>
       </c>
@@ -6019,14 +6049,14 @@
       <c r="C125" s="15" t="s">
         <v>298</v>
       </c>
-      <c r="D125" t="s">
-        <v>299</v>
+      <c r="D125" s="36" t="s">
+        <v>511</v>
       </c>
       <c r="F125" s="27" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="126" spans="1:26">
+    <row r="126" spans="1:26" ht="39">
       <c r="A126" s="15" t="s">
         <v>110</v>
       </c>
@@ -6036,8 +6066,8 @@
       <c r="C126" s="15" t="s">
         <v>302</v>
       </c>
-      <c r="D126" s="14" t="s">
-        <v>303</v>
+      <c r="D126" s="18" t="s">
+        <v>512</v>
       </c>
       <c r="F126" s="27" t="s">
         <v>304</v>
@@ -6077,7 +6107,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="129" spans="1:1024">
+    <row r="129" spans="1:1024" ht="65">
       <c r="A129" s="15" t="s">
         <v>110</v>
       </c>
@@ -6087,14 +6117,14 @@
       <c r="C129" s="15" t="s">
         <v>314</v>
       </c>
-      <c r="D129" s="14" t="s">
-        <v>315</v>
+      <c r="D129" s="18" t="s">
+        <v>513</v>
       </c>
       <c r="F129" s="27" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="130" spans="1:1024">
+    <row r="130" spans="1:1024" ht="52">
       <c r="A130" s="15" t="s">
         <v>110</v>
       </c>
@@ -6104,8 +6134,8 @@
       <c r="C130" s="15" t="s">
         <v>318</v>
       </c>
-      <c r="D130" s="14" t="s">
-        <v>319</v>
+      <c r="D130" s="18" t="s">
+        <v>514</v>
       </c>
       <c r="F130" s="27" t="s">
         <v>320</v>
@@ -6389,10 +6419,10 @@
         <v>346</v>
       </c>
       <c r="D147" s="14" t="s">
+        <v>515</v>
+      </c>
+      <c r="F147" s="14" t="s">
         <v>364</v>
-      </c>
-      <c r="F147" s="14" t="s">
-        <v>365</v>
       </c>
       <c r="AMJ147"/>
     </row>
@@ -6401,16 +6431,16 @@
         <v>110</v>
       </c>
       <c r="B148" t="s">
+        <v>365</v>
+      </c>
+      <c r="C148" s="26" t="s">
         <v>366</v>
       </c>
-      <c r="C148" s="26" t="s">
+      <c r="D148" s="26" t="s">
         <v>367</v>
       </c>
-      <c r="D148" s="26" t="s">
+      <c r="F148" t="s">
         <v>368</v>
-      </c>
-      <c r="F148" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="149" spans="1:1024">
@@ -6418,16 +6448,16 @@
         <v>110</v>
       </c>
       <c r="B149" t="s">
+        <v>369</v>
+      </c>
+      <c r="C149" s="26" t="s">
         <v>370</v>
       </c>
-      <c r="C149" s="26" t="s">
+      <c r="D149" s="26" t="s">
         <v>371</v>
       </c>
-      <c r="D149" s="26" t="s">
+      <c r="F149" t="s">
         <v>372</v>
-      </c>
-      <c r="F149" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="150" spans="1:1024">
@@ -6435,16 +6465,16 @@
         <v>110</v>
       </c>
       <c r="B150" t="s">
+        <v>373</v>
+      </c>
+      <c r="C150" s="26" t="s">
         <v>374</v>
       </c>
-      <c r="C150" s="26" t="s">
+      <c r="D150" s="26" t="s">
         <v>375</v>
       </c>
-      <c r="D150" s="26" t="s">
+      <c r="F150" t="s">
         <v>376</v>
-      </c>
-      <c r="F150" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="151" spans="1:1024">
@@ -6452,16 +6482,16 @@
         <v>110</v>
       </c>
       <c r="B151" t="s">
+        <v>377</v>
+      </c>
+      <c r="C151" s="26" t="s">
         <v>378</v>
       </c>
-      <c r="C151" s="26" t="s">
+      <c r="D151" s="26" t="s">
         <v>379</v>
       </c>
-      <c r="D151" s="26" t="s">
+      <c r="F151" t="s">
         <v>380</v>
-      </c>
-      <c r="F151" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="152" spans="1:1024">
@@ -6469,16 +6499,16 @@
         <v>110</v>
       </c>
       <c r="B152" t="s">
+        <v>381</v>
+      </c>
+      <c r="C152" s="26" t="s">
         <v>382</v>
       </c>
-      <c r="C152" s="26" t="s">
+      <c r="D152" s="26" t="s">
         <v>383</v>
       </c>
-      <c r="D152" s="26" t="s">
+      <c r="F152" t="s">
         <v>384</v>
-      </c>
-      <c r="F152" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="153" spans="1:1024">
@@ -6486,16 +6516,16 @@
         <v>110</v>
       </c>
       <c r="B153" t="s">
+        <v>385</v>
+      </c>
+      <c r="C153" s="26" t="s">
         <v>386</v>
       </c>
-      <c r="C153" s="26" t="s">
+      <c r="D153" s="26" t="s">
         <v>387</v>
       </c>
-      <c r="D153" s="26" t="s">
+      <c r="F153" t="s">
         <v>388</v>
-      </c>
-      <c r="F153" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="154" spans="1:1024">
@@ -6503,16 +6533,16 @@
         <v>110</v>
       </c>
       <c r="B154" t="s">
+        <v>389</v>
+      </c>
+      <c r="C154" s="26" t="s">
         <v>390</v>
       </c>
-      <c r="C154" s="26" t="s">
+      <c r="D154" s="26" t="s">
         <v>391</v>
       </c>
-      <c r="D154" s="26" t="s">
+      <c r="F154" t="s">
         <v>392</v>
-      </c>
-      <c r="F154" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="155" spans="1:1024" s="15" customFormat="1">
@@ -6529,13 +6559,13 @@
         <v>106</v>
       </c>
       <c r="B156" s="15" t="s">
+        <v>393</v>
+      </c>
+      <c r="C156" t="s">
         <v>394</v>
       </c>
-      <c r="C156" t="s">
+      <c r="D156" t="s">
         <v>395</v>
-      </c>
-      <c r="D156" t="s">
-        <v>396</v>
       </c>
       <c r="G156" t="s">
         <v>245</v>
@@ -6547,16 +6577,16 @@
         <v>110</v>
       </c>
       <c r="B157" s="18" t="s">
+        <v>396</v>
+      </c>
+      <c r="C157" s="18" t="s">
         <v>397</v>
       </c>
-      <c r="C157" s="18" t="s">
+      <c r="D157" s="20" t="s">
         <v>398</v>
       </c>
-      <c r="D157" s="20" t="s">
+      <c r="F157" s="18" t="s">
         <v>399</v>
-      </c>
-      <c r="F157" s="18" t="s">
-        <v>400</v>
       </c>
       <c r="G157" s="18"/>
       <c r="H157" s="18"/>
@@ -6584,19 +6614,19 @@
         <v>110</v>
       </c>
       <c r="B158" s="18" t="s">
+        <v>400</v>
+      </c>
+      <c r="C158" s="18" t="s">
         <v>401</v>
       </c>
-      <c r="C158" s="18" t="s">
+      <c r="D158" s="29" t="s">
         <v>402</v>
       </c>
-      <c r="D158" s="29" t="s">
+      <c r="F158" s="19" t="s">
         <v>403</v>
       </c>
-      <c r="F158" s="19" t="s">
+      <c r="G158" s="18" t="s">
         <v>404</v>
-      </c>
-      <c r="G158" s="18" t="s">
-        <v>405</v>
       </c>
       <c r="H158" s="18"/>
       <c r="I158" s="18"/>
@@ -6618,24 +6648,24 @@
       <c r="Y158" s="18"/>
       <c r="AMJ158"/>
     </row>
-    <row r="159" spans="1:1024" s="15" customFormat="1" ht="57">
+    <row r="159" spans="1:1024" s="15" customFormat="1" ht="42.75">
       <c r="A159" s="18" t="s">
         <v>110</v>
       </c>
       <c r="B159" s="18" t="s">
+        <v>405</v>
+      </c>
+      <c r="C159" s="18" t="s">
         <v>406</v>
       </c>
-      <c r="C159" s="18" t="s">
+      <c r="D159" s="18" t="s">
         <v>407</v>
       </c>
-      <c r="D159" s="18" t="s">
+      <c r="F159" s="30" t="s">
         <v>408</v>
       </c>
-      <c r="F159" s="30" t="s">
-        <v>409</v>
-      </c>
       <c r="G159" s="18" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="H159" s="18"/>
       <c r="I159" s="18"/>
@@ -6661,13 +6691,13 @@
         <v>110</v>
       </c>
       <c r="B160" s="15" t="s">
+        <v>409</v>
+      </c>
+      <c r="C160" t="s">
         <v>410</v>
       </c>
-      <c r="C160" t="s">
+      <c r="D160" t="s">
         <v>411</v>
-      </c>
-      <c r="D160" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="161" spans="1:1024">
@@ -6675,7 +6705,7 @@
         <v>114</v>
       </c>
       <c r="B161" s="15" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="J161" s="18"/>
     </row>
@@ -6684,7 +6714,7 @@
         <v>42</v>
       </c>
       <c r="B162" s="18" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C162" s="18"/>
       <c r="D162" s="18"/>
@@ -6694,7 +6724,7 @@
       <c r="H162" s="18"/>
       <c r="I162" s="18"/>
       <c r="L162" s="18" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="M162" s="18"/>
       <c r="N162" s="18"/>
@@ -6717,10 +6747,10 @@
         <v>42</v>
       </c>
       <c r="B163" s="28" t="s">
+        <v>414</v>
+      </c>
+      <c r="L163" s="28" t="s">
         <v>415</v>
-      </c>
-      <c r="L163" s="28" t="s">
-        <v>416</v>
       </c>
       <c r="AMJ163"/>
     </row>
@@ -6729,10 +6759,10 @@
         <v>42</v>
       </c>
       <c r="B164" s="28" t="s">
+        <v>416</v>
+      </c>
+      <c r="L164" s="28" t="s">
         <v>417</v>
-      </c>
-      <c r="L164" s="28" t="s">
-        <v>418</v>
       </c>
       <c r="AMJ164"/>
     </row>
@@ -6741,10 +6771,10 @@
         <v>42</v>
       </c>
       <c r="B165" s="28" t="s">
+        <v>418</v>
+      </c>
+      <c r="L165" s="28" t="s">
         <v>419</v>
-      </c>
-      <c r="L165" s="28" t="s">
-        <v>420</v>
       </c>
       <c r="AMJ165"/>
     </row>
@@ -6771,7 +6801,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1">
       <c r="A1" s="31" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B1" s="31" t="s">
         <v>1</v>
@@ -6812,7 +6842,7 @@
         <v>237</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C2" s="32" t="s">
         <v>247</v>
@@ -6962,7 +6992,7 @@
         <v>263</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E6" s="18"/>
       <c r="F6" s="18"/>
@@ -7532,7 +7562,7 @@
         <v>237</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C22" s="20" t="s">
         <v>326</v>
@@ -7676,7 +7706,7 @@
         <v>237</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C26" s="20" t="s">
         <v>342</v>
@@ -7712,13 +7742,13 @@
         <v>237</v>
       </c>
       <c r="B27" s="18" t="s">
+        <v>425</v>
+      </c>
+      <c r="C27" s="20" t="s">
         <v>426</v>
       </c>
-      <c r="C27" s="20" t="s">
+      <c r="D27" s="14" t="s">
         <v>427</v>
-      </c>
-      <c r="D27" s="14" t="s">
-        <v>428</v>
       </c>
       <c r="E27" s="18"/>
       <c r="F27" s="18"/>
@@ -7745,142 +7775,142 @@
     </row>
     <row r="28" spans="1:26" ht="15.75" customHeight="1">
       <c r="A28" s="15" t="s">
+        <v>428</v>
+      </c>
+      <c r="B28" s="15" t="s">
         <v>429</v>
       </c>
-      <c r="B28" s="15" t="s">
+      <c r="C28" s="15" t="s">
         <v>430</v>
       </c>
-      <c r="C28" s="15" t="s">
+      <c r="D28" s="14" t="s">
         <v>431</v>
-      </c>
-      <c r="D28" s="14" t="s">
-        <v>432</v>
       </c>
     </row>
     <row r="29" spans="1:26" ht="15.75" customHeight="1">
       <c r="A29" s="15" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B29" s="15" t="s">
+        <v>432</v>
+      </c>
+      <c r="C29" s="15" t="s">
         <v>433</v>
       </c>
-      <c r="C29" s="15" t="s">
+      <c r="D29" s="14" t="s">
         <v>434</v>
-      </c>
-      <c r="D29" s="14" t="s">
-        <v>435</v>
       </c>
     </row>
     <row r="30" spans="1:26" ht="15.75" customHeight="1">
       <c r="A30" s="15" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B30" s="15" t="s">
+        <v>435</v>
+      </c>
+      <c r="C30" s="15" t="s">
         <v>436</v>
       </c>
-      <c r="C30" s="15" t="s">
+      <c r="D30" s="14" t="s">
         <v>437</v>
-      </c>
-      <c r="D30" s="14" t="s">
-        <v>438</v>
       </c>
     </row>
     <row r="31" spans="1:26" ht="15.75" customHeight="1">
       <c r="A31" s="15" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B31" s="15" t="s">
+        <v>438</v>
+      </c>
+      <c r="C31" s="15" t="s">
         <v>439</v>
       </c>
-      <c r="C31" s="15" t="s">
+      <c r="D31" s="14" t="s">
         <v>440</v>
-      </c>
-      <c r="D31" s="14" t="s">
-        <v>441</v>
       </c>
     </row>
     <row r="32" spans="1:26" ht="15.75" customHeight="1">
       <c r="A32" s="15" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B32" s="15" t="s">
+        <v>441</v>
+      </c>
+      <c r="C32" s="15" t="s">
         <v>442</v>
       </c>
-      <c r="C32" s="15" t="s">
+      <c r="D32" s="14" t="s">
         <v>443</v>
-      </c>
-      <c r="D32" s="14" t="s">
-        <v>444</v>
       </c>
     </row>
     <row r="33" spans="1:26" ht="15.75" customHeight="1">
       <c r="A33" s="15" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B33" s="15" t="s">
+        <v>444</v>
+      </c>
+      <c r="C33" s="15" t="s">
         <v>445</v>
       </c>
-      <c r="C33" s="15" t="s">
+      <c r="D33" s="14" t="s">
         <v>446</v>
-      </c>
-      <c r="D33" s="14" t="s">
-        <v>447</v>
       </c>
     </row>
     <row r="34" spans="1:26" ht="15.75" customHeight="1">
       <c r="A34" s="15" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B34" s="14" t="s">
+        <v>447</v>
+      </c>
+      <c r="C34" s="15" t="s">
         <v>448</v>
       </c>
-      <c r="C34" s="15" t="s">
+      <c r="D34" s="14" t="s">
         <v>449</v>
-      </c>
-      <c r="D34" s="14" t="s">
-        <v>450</v>
       </c>
     </row>
     <row r="35" spans="1:26" ht="15.75" customHeight="1">
       <c r="A35" s="15" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B35" s="14" t="s">
+        <v>425</v>
+      </c>
+      <c r="C35" s="15" t="s">
         <v>426</v>
       </c>
-      <c r="C35" s="15" t="s">
-        <v>427</v>
-      </c>
       <c r="D35" s="15" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="36" spans="1:26" ht="15.75" customHeight="1">
       <c r="A36" s="14" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B36" s="14" t="s">
         <v>160</v>
       </c>
       <c r="C36" s="14" t="s">
+        <v>451</v>
+      </c>
+      <c r="D36" s="14" t="s">
         <v>452</v>
-      </c>
-      <c r="D36" s="14" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="37" spans="1:26">
       <c r="A37" s="14" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B37" s="14" t="s">
+        <v>453</v>
+      </c>
+      <c r="C37" s="14" t="s">
         <v>454</v>
       </c>
-      <c r="C37" s="14" t="s">
+      <c r="D37" s="14" t="s">
         <v>455</v>
-      </c>
-      <c r="D37" s="14" t="s">
-        <v>456</v>
       </c>
     </row>
     <row r="38" spans="1:26">
@@ -7888,13 +7918,13 @@
         <v>202</v>
       </c>
       <c r="B38" s="18" t="s">
+        <v>456</v>
+      </c>
+      <c r="C38" s="18" t="s">
         <v>457</v>
       </c>
-      <c r="C38" s="18" t="s">
+      <c r="D38" s="20" t="s">
         <v>458</v>
-      </c>
-      <c r="D38" s="20" t="s">
-        <v>459</v>
       </c>
       <c r="E38" s="18"/>
       <c r="F38" s="18"/>
@@ -7924,13 +7954,13 @@
         <v>202</v>
       </c>
       <c r="B39" s="18" t="s">
+        <v>459</v>
+      </c>
+      <c r="C39" s="18" t="s">
         <v>460</v>
       </c>
-      <c r="C39" s="18" t="s">
+      <c r="D39" s="18" t="s">
         <v>461</v>
-      </c>
-      <c r="D39" s="18" t="s">
-        <v>462</v>
       </c>
       <c r="E39" s="18"/>
       <c r="F39" s="18"/>
@@ -7960,13 +7990,13 @@
         <v>202</v>
       </c>
       <c r="B40" s="18" t="s">
+        <v>462</v>
+      </c>
+      <c r="C40" s="18" t="s">
         <v>463</v>
       </c>
-      <c r="C40" s="18" t="s">
+      <c r="D40" s="18" t="s">
         <v>464</v>
-      </c>
-      <c r="D40" s="18" t="s">
-        <v>465</v>
       </c>
       <c r="E40" s="18"/>
       <c r="F40" s="18"/>
@@ -7996,13 +8026,13 @@
         <v>202</v>
       </c>
       <c r="B41" s="18" t="s">
+        <v>465</v>
+      </c>
+      <c r="C41" s="18" t="s">
         <v>466</v>
       </c>
-      <c r="C41" s="18" t="s">
+      <c r="D41" s="20" t="s">
         <v>467</v>
-      </c>
-      <c r="D41" s="20" t="s">
-        <v>468</v>
       </c>
       <c r="E41" s="18"/>
       <c r="F41" s="18"/>
@@ -8032,13 +8062,13 @@
         <v>202</v>
       </c>
       <c r="B42" s="18" t="s">
+        <v>468</v>
+      </c>
+      <c r="C42" s="18" t="s">
         <v>469</v>
       </c>
-      <c r="C42" s="18" t="s">
+      <c r="D42" s="18" t="s">
         <v>470</v>
-      </c>
-      <c r="D42" s="18" t="s">
-        <v>471</v>
       </c>
       <c r="E42" s="18"/>
       <c r="F42" s="18"/>
@@ -8068,13 +8098,13 @@
         <v>202</v>
       </c>
       <c r="B43" s="18" t="s">
+        <v>471</v>
+      </c>
+      <c r="C43" s="18" t="s">
         <v>472</v>
       </c>
-      <c r="C43" s="18" t="s">
+      <c r="D43" s="20" t="s">
         <v>473</v>
-      </c>
-      <c r="D43" s="20" t="s">
-        <v>474</v>
       </c>
       <c r="E43" s="18"/>
       <c r="F43" s="18"/>
@@ -8104,13 +8134,13 @@
         <v>202</v>
       </c>
       <c r="B44" s="18" t="s">
+        <v>474</v>
+      </c>
+      <c r="C44" s="18" t="s">
         <v>475</v>
       </c>
-      <c r="C44" s="18" t="s">
+      <c r="D44" s="20" t="s">
         <v>476</v>
-      </c>
-      <c r="D44" s="20" t="s">
-        <v>477</v>
       </c>
       <c r="E44" s="18"/>
       <c r="F44" s="18"/>
@@ -8140,13 +8170,13 @@
         <v>202</v>
       </c>
       <c r="B45" s="18" t="s">
+        <v>477</v>
+      </c>
+      <c r="C45" s="18" t="s">
         <v>478</v>
       </c>
-      <c r="C45" s="18" t="s">
+      <c r="D45" s="20" t="s">
         <v>479</v>
-      </c>
-      <c r="D45" s="20" t="s">
-        <v>480</v>
       </c>
       <c r="E45" s="18"/>
       <c r="F45" s="18"/>
@@ -8176,13 +8206,13 @@
         <v>202</v>
       </c>
       <c r="B46" s="18" t="s">
+        <v>480</v>
+      </c>
+      <c r="C46" s="18" t="s">
         <v>481</v>
       </c>
-      <c r="C46" s="18" t="s">
+      <c r="D46" s="20" t="s">
         <v>482</v>
-      </c>
-      <c r="D46" s="20" t="s">
-        <v>483</v>
       </c>
       <c r="E46" s="18"/>
       <c r="F46" s="18"/>
@@ -8212,13 +8242,13 @@
         <v>202</v>
       </c>
       <c r="B47" s="18" t="s">
+        <v>483</v>
+      </c>
+      <c r="C47" s="18" t="s">
         <v>484</v>
       </c>
-      <c r="C47" s="18" t="s">
+      <c r="D47" s="20" t="s">
         <v>485</v>
-      </c>
-      <c r="D47" s="20" t="s">
-        <v>486</v>
       </c>
       <c r="E47" s="18"/>
       <c r="F47" s="18"/>
@@ -8248,13 +8278,13 @@
         <v>202</v>
       </c>
       <c r="B48" s="18" t="s">
+        <v>486</v>
+      </c>
+      <c r="C48" s="18" t="s">
         <v>487</v>
       </c>
-      <c r="C48" s="18" t="s">
+      <c r="D48" s="20" t="s">
         <v>488</v>
-      </c>
-      <c r="D48" s="20" t="s">
-        <v>489</v>
       </c>
       <c r="E48" s="18"/>
       <c r="F48" s="18"/>
@@ -8284,13 +8314,13 @@
         <v>202</v>
       </c>
       <c r="B49" s="18" t="s">
+        <v>489</v>
+      </c>
+      <c r="C49" s="18" t="s">
         <v>490</v>
       </c>
-      <c r="C49" s="18" t="s">
+      <c r="D49" s="20" t="s">
         <v>491</v>
-      </c>
-      <c r="D49" s="20" t="s">
-        <v>492</v>
       </c>
       <c r="E49" s="18"/>
       <c r="F49" s="18"/>
@@ -8320,13 +8350,13 @@
         <v>202</v>
       </c>
       <c r="B50" s="18" t="s">
+        <v>492</v>
+      </c>
+      <c r="C50" s="18" t="s">
         <v>493</v>
       </c>
-      <c r="C50" s="18" t="s">
+      <c r="D50" s="20" t="s">
         <v>494</v>
-      </c>
-      <c r="D50" s="20" t="s">
-        <v>495</v>
       </c>
       <c r="E50" s="18"/>
       <c r="F50" s="18"/>
@@ -8356,13 +8386,13 @@
         <v>202</v>
       </c>
       <c r="B51" s="18" t="s">
+        <v>425</v>
+      </c>
+      <c r="C51" s="18" t="s">
         <v>426</v>
       </c>
-      <c r="C51" s="18" t="s">
+      <c r="D51" s="20" t="s">
         <v>427</v>
-      </c>
-      <c r="D51" s="20" t="s">
-        <v>428</v>
       </c>
       <c r="E51" s="18"/>
       <c r="F51" s="18"/>
@@ -8405,22 +8435,22 @@
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1">
       <c r="A1" s="31" t="s">
+        <v>495</v>
+      </c>
+      <c r="B1" s="31" t="s">
         <v>496</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="C1" s="31" t="s">
         <v>497</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="D1" s="31" t="s">
         <v>498</v>
       </c>
-      <c r="D1" s="31" t="s">
+      <c r="E1" s="31" t="s">
         <v>499</v>
       </c>
-      <c r="E1" s="31" t="s">
+      <c r="F1" s="31" t="s">
         <v>500</v>
-      </c>
-      <c r="F1" s="31" t="s">
-        <v>501</v>
       </c>
       <c r="G1" s="15"/>
       <c r="H1" s="15"/>
@@ -8445,19 +8475,19 @@
     </row>
     <row r="2" spans="1:26" ht="15.75" customHeight="1">
       <c r="A2" s="25" t="s">
+        <v>505</v>
+      </c>
+      <c r="B2" s="25" t="s">
         <v>506</v>
       </c>
-      <c r="B2" s="25" t="s">
-        <v>507</v>
-      </c>
       <c r="C2" s="33" t="s">
+        <v>501</v>
+      </c>
+      <c r="D2" s="25" t="s">
         <v>502</v>
       </c>
-      <c r="D2" s="25" t="s">
+      <c r="E2" s="25" t="s">
         <v>503</v>
-      </c>
-      <c r="E2" s="25" t="s">
-        <v>504</v>
       </c>
       <c r="F2" s="25"/>
       <c r="G2" s="15"/>

</xml_diff>

<commit_message>
removed unsupported Array.prototype.flat which made the app clash
</commit_message>
<xml_diff>
--- a/forms/app/pregnancy_counselling.xlsx
+++ b/forms/app/pregnancy_counselling.xlsx
@@ -796,10 +796,10 @@
     <t xml:space="preserve">risk_factors</t>
   </si>
   <si>
-    <t xml:space="preserve">Which pregnancy risk factors do you remember?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Je unakumbuka sababu zipi za hatari za ujauzito? </t>
+    <t xml:space="preserve">Which pregnancy risk factors among those which we discussed in previous visit do you remember?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je unakumbuka  hali hatarishi zipi za ujauzito katika zile tulizojadili katika tembeleo lililopita?</t>
   </si>
   <si>
     <t xml:space="preserve">${high_risk_manual}  = "true" </t>
@@ -1123,7 +1123,7 @@
     <t xml:space="preserve">Kuepuka kula baadhi ya vyakula </t>
   </si>
   <si>
-    <t xml:space="preserve">not(selected(${risk_factors},'nutrition_restrictions')) and contains(${risk_factor_names}, 'nutrition')</t>
+    <t xml:space="preserve">not(selected(${risk_factors},'nutrition_restrictions')) and contains(${risk_factor_names}, 'nutrition_restriction')</t>
   </si>
   <si>
     <t xml:space="preserve">mitigation_strategy</t>
@@ -1894,11 +1894,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5437,14 +5437,14 @@
       <c r="Y108" s="15"/>
       <c r="Z108" s="15"/>
     </row>
-    <row r="109" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="15" t="s">
         <v>239</v>
       </c>
       <c r="B109" s="15" t="s">
         <v>240</v>
       </c>
-      <c r="C109" s="25" t="s">
+      <c r="C109" s="17" t="s">
         <v>241</v>
       </c>
       <c r="D109" s="15" t="s">
@@ -5458,13 +5458,13 @@
       </c>
       <c r="G109" s="15"/>
       <c r="H109" s="15"/>
-      <c r="I109" s="26" t="s">
+      <c r="I109" s="25" t="s">
         <v>209</v>
       </c>
-      <c r="J109" s="26" t="s">
+      <c r="J109" s="25" t="s">
         <v>244</v>
       </c>
-      <c r="K109" s="26" t="s">
+      <c r="K109" s="25" t="s">
         <v>211</v>
       </c>
       <c r="L109" s="15"/>
@@ -5560,7 +5560,7 @@
       <c r="B112" s="15" t="s">
         <v>249</v>
       </c>
-      <c r="C112" s="25" t="s">
+      <c r="C112" s="26" t="s">
         <v>250</v>
       </c>
       <c r="D112" s="14" t="s">
@@ -6079,13 +6079,13 @@
       <c r="E140" s="14" t="s">
         <v>163</v>
       </c>
-      <c r="I140" s="26" t="s">
+      <c r="I140" s="25" t="s">
         <v>209</v>
       </c>
-      <c r="J140" s="26" t="s">
+      <c r="J140" s="25" t="s">
         <v>244</v>
       </c>
-      <c r="K140" s="26" t="s">
+      <c r="K140" s="25" t="s">
         <v>211</v>
       </c>
       <c r="M140" s="14" t="s">
@@ -6150,7 +6150,7 @@
       <c r="E144" s="14" t="s">
         <v>163</v>
       </c>
-      <c r="I144" s="26" t="s">
+      <c r="I144" s="25" t="s">
         <v>209</v>
       </c>
       <c r="M144" s="14" t="s">
@@ -6203,10 +6203,10 @@
       <c r="B148" s="0" t="s">
         <v>370</v>
       </c>
-      <c r="C148" s="26" t="s">
+      <c r="C148" s="25" t="s">
         <v>371</v>
       </c>
-      <c r="D148" s="26" t="s">
+      <c r="D148" s="25" t="s">
         <v>372</v>
       </c>
       <c r="F148" s="0" t="s">
@@ -6220,10 +6220,10 @@
       <c r="B149" s="0" t="s">
         <v>374</v>
       </c>
-      <c r="C149" s="26" t="s">
+      <c r="C149" s="25" t="s">
         <v>375</v>
       </c>
-      <c r="D149" s="26" t="s">
+      <c r="D149" s="25" t="s">
         <v>376</v>
       </c>
       <c r="F149" s="0" t="s">
@@ -6237,10 +6237,10 @@
       <c r="B150" s="0" t="s">
         <v>378</v>
       </c>
-      <c r="C150" s="26" t="s">
+      <c r="C150" s="25" t="s">
         <v>379</v>
       </c>
-      <c r="D150" s="26" t="s">
+      <c r="D150" s="25" t="s">
         <v>380</v>
       </c>
       <c r="F150" s="0" t="s">
@@ -6254,10 +6254,10 @@
       <c r="B151" s="0" t="s">
         <v>382</v>
       </c>
-      <c r="C151" s="26" t="s">
+      <c r="C151" s="25" t="s">
         <v>383</v>
       </c>
-      <c r="D151" s="26" t="s">
+      <c r="D151" s="25" t="s">
         <v>384</v>
       </c>
       <c r="F151" s="0" t="s">
@@ -6271,10 +6271,10 @@
       <c r="B152" s="0" t="s">
         <v>386</v>
       </c>
-      <c r="C152" s="26" t="s">
+      <c r="C152" s="25" t="s">
         <v>387</v>
       </c>
-      <c r="D152" s="26" t="s">
+      <c r="D152" s="25" t="s">
         <v>388</v>
       </c>
       <c r="F152" s="0" t="s">
@@ -6288,10 +6288,10 @@
       <c r="B153" s="0" t="s">
         <v>390</v>
       </c>
-      <c r="C153" s="26" t="s">
+      <c r="C153" s="25" t="s">
         <v>391</v>
       </c>
-      <c r="D153" s="26" t="s">
+      <c r="D153" s="25" t="s">
         <v>392</v>
       </c>
       <c r="F153" s="0" t="s">
@@ -6305,10 +6305,10 @@
       <c r="B154" s="0" t="s">
         <v>394</v>
       </c>
-      <c r="C154" s="26" t="s">
+      <c r="C154" s="25" t="s">
         <v>395</v>
       </c>
-      <c r="D154" s="26" t="s">
+      <c r="D154" s="25" t="s">
         <v>396</v>
       </c>
       <c r="F154" s="0" t="s">
@@ -6562,9 +6562,9 @@
   <dimension ref="A1:Z51"/>
   <sheetFormatPr defaultRowHeight="13" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="72.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="72.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="53.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="5" style="0" width="14.41"/>
   </cols>
@@ -8252,22 +8252,22 @@
       <c r="Z1" s="15"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="26" t="s">
         <v>511</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="26" t="s">
         <v>512</v>
       </c>
       <c r="C2" s="32" t="s">
         <v>513</v>
       </c>
-      <c r="D2" s="25" t="s">
+      <c r="D2" s="26" t="s">
         <v>514</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="E2" s="26" t="s">
         <v>515</v>
       </c>
-      <c r="F2" s="25"/>
+      <c r="F2" s="26"/>
       <c r="G2" s="15"/>
       <c r="H2" s="15"/>
       <c r="I2" s="15"/>

</xml_diff>